<commit_message>
plot anomaly detection: x-label to seconds instead of index + Hz
</commit_message>
<xml_diff>
--- a/Fragebogen/Fragebogen_Auswertung_quantitativ.xlsx
+++ b/Fragebogen/Fragebogen_Auswertung_quantitativ.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jonas\Desktop\Uni\BA\Durchführung\Datenanalyse\Fragebogen\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Backups\Uni\BA\Durchführung\Datenanalyse\Fragebogen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDA87379-714F-480E-9EAB-70AE1AE2FE76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92D5F950-30FE-49C5-9A10-0015ED04C329}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38510" yWindow="-3590" windowWidth="38620" windowHeight="21220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="25">
   <si>
     <t>TeilnehmerIn</t>
   </si>
@@ -129,9 +129,6 @@
   </si>
   <si>
     <t>Standartabweichung</t>
-  </si>
-  <si>
-    <t>revidieren</t>
   </si>
 </sst>
 </file>
@@ -467,13 +464,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:T12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:T11"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.88671875" customWidth="1"/>
+    <col min="1" max="1" width="18.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="230.4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:20" ht="255" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -535,7 +532,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -569,18 +566,10 @@
       <c r="K2" s="3">
         <v>4</v>
       </c>
-      <c r="L2" s="3">
-        <v>1</v>
-      </c>
-      <c r="M2" s="3">
-        <v>1</v>
-      </c>
-      <c r="N2" s="3">
-        <v>1</v>
-      </c>
-      <c r="O2" s="3">
-        <v>1</v>
-      </c>
+      <c r="L2" s="3"/>
+      <c r="M2" s="3"/>
+      <c r="N2" s="3"/>
+      <c r="O2" s="3"/>
       <c r="P2" s="3">
         <v>3</v>
       </c>
@@ -595,7 +584,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -632,15 +621,9 @@
       <c r="L3" s="3">
         <v>4</v>
       </c>
-      <c r="M3" s="3">
-        <v>1</v>
-      </c>
-      <c r="N3" s="3">
-        <v>1</v>
-      </c>
-      <c r="O3" s="3">
-        <v>1</v>
-      </c>
+      <c r="M3" s="3"/>
+      <c r="N3" s="3"/>
+      <c r="O3" s="3"/>
       <c r="P3" s="3">
         <v>2</v>
       </c>
@@ -657,7 +640,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -691,18 +674,10 @@
       <c r="K4" s="3">
         <v>3</v>
       </c>
-      <c r="L4" s="3">
-        <v>1</v>
-      </c>
-      <c r="M4" s="3">
-        <v>1</v>
-      </c>
-      <c r="N4" s="3">
-        <v>1</v>
-      </c>
-      <c r="O4" s="3">
-        <v>1</v>
-      </c>
+      <c r="L4" s="3"/>
+      <c r="M4" s="3"/>
+      <c r="N4" s="3"/>
+      <c r="O4" s="3"/>
       <c r="P4" s="3">
         <v>4</v>
       </c>
@@ -717,7 +692,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -751,18 +726,14 @@
       <c r="K5" s="3">
         <v>4</v>
       </c>
-      <c r="L5" s="3">
-        <v>1</v>
-      </c>
+      <c r="L5" s="3"/>
       <c r="M5" s="3">
         <v>3</v>
       </c>
       <c r="N5" s="3">
         <v>3</v>
       </c>
-      <c r="O5" s="3">
-        <v>1</v>
-      </c>
+      <c r="O5" s="3"/>
       <c r="P5" s="3">
         <v>4</v>
       </c>
@@ -779,7 +750,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -813,18 +784,10 @@
       <c r="K6" s="3">
         <v>4</v>
       </c>
-      <c r="L6" s="3">
-        <v>1</v>
-      </c>
-      <c r="M6" s="3">
-        <v>1</v>
-      </c>
-      <c r="N6" s="3">
-        <v>1</v>
-      </c>
-      <c r="O6" s="3">
-        <v>1</v>
-      </c>
+      <c r="L6" s="3"/>
+      <c r="M6" s="3"/>
+      <c r="N6" s="3"/>
+      <c r="O6" s="3"/>
       <c r="P6" s="3">
         <v>3</v>
       </c>
@@ -841,7 +804,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -875,15 +838,11 @@
       <c r="K7" s="3">
         <v>2</v>
       </c>
-      <c r="L7" s="3">
-        <v>1</v>
-      </c>
+      <c r="L7" s="3"/>
       <c r="M7" s="3">
         <v>4</v>
       </c>
-      <c r="N7" s="3">
-        <v>1</v>
-      </c>
+      <c r="N7" s="3"/>
       <c r="O7" s="3">
         <v>4</v>
       </c>
@@ -903,7 +862,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -937,15 +896,11 @@
       <c r="K8" s="3">
         <v>4</v>
       </c>
-      <c r="L8" s="3">
-        <v>1</v>
-      </c>
+      <c r="L8" s="3"/>
       <c r="M8" s="3">
         <v>3</v>
       </c>
-      <c r="N8" s="3">
-        <v>1</v>
-      </c>
+      <c r="N8" s="3"/>
       <c r="O8" s="3">
         <v>3</v>
       </c>
@@ -965,7 +920,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:20" ht="72" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:20" ht="75" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -1025,7 +980,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
         <v>23</v>
       </c>
@@ -1059,19 +1014,19 @@
       </c>
       <c r="L10" s="4">
         <f t="shared" si="1"/>
-        <v>1.375</v>
+        <v>2.5</v>
       </c>
       <c r="M10" s="4">
         <f t="shared" si="1"/>
-        <v>1.875</v>
+        <v>2.75</v>
       </c>
       <c r="N10" s="4">
         <f t="shared" si="1"/>
-        <v>1.25</v>
+        <v>2</v>
       </c>
       <c r="O10" s="4">
         <f t="shared" si="1"/>
-        <v>1.625</v>
+        <v>2.6666666666666665</v>
       </c>
       <c r="P10" s="4">
         <f t="shared" si="1"/>
@@ -1094,7 +1049,7 @@
         <v>3.75</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>24</v>
       </c>
@@ -1128,19 +1083,19 @@
       </c>
       <c r="L11" s="4">
         <f t="shared" si="3"/>
-        <v>0.99215674164922152</v>
+        <v>1.5</v>
       </c>
       <c r="M11" s="4">
         <f t="shared" si="3"/>
-        <v>1.165922381636102</v>
+        <v>1.0897247358851685</v>
       </c>
       <c r="N11" s="4">
         <f t="shared" si="3"/>
-        <v>0.66143782776614768</v>
+        <v>1</v>
       </c>
       <c r="O11" s="4">
         <f t="shared" si="3"/>
-        <v>1.1110243021644486</v>
+        <v>1.247219128924647</v>
       </c>
       <c r="P11" s="4">
         <f t="shared" si="3"/>
@@ -1161,17 +1116,6 @@
       <c r="T11" s="4">
         <f t="shared" si="3"/>
         <v>0.82915619758884995</v>
-      </c>
-    </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="L12" t="s">
-        <v>25</v>
-      </c>
-      <c r="M12" t="s">
-        <v>25</v>
-      </c>
-      <c r="N12" t="s">
-        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>